<commit_message>
Added BD Male External Catheter
U5
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dvagov-my.sharepoint.com/personal/bernard_chan_va_gov/Documents/Microsoft Teams Chat Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="11_87A73CECC8785890643FEBC9776139824E07390D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DC67227-D43E-4D83-9019-D21FCC478F9F}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="11_87A73CECC8785890643FEBC9776139824E07390D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBDFB50C-05FA-4165-95BE-D76492117E0F}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2046" uniqueCount="869">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2056" uniqueCount="873">
   <si>
     <t>category</t>
   </si>
@@ -2643,6 +2643,18 @@
   </si>
   <si>
     <t>Washed and reused ~3 days, so one per day.</t>
+  </si>
+  <si>
+    <t>Male External Catheter BD UltraFlex</t>
+  </si>
+  <si>
+    <t>Medium 29mm</t>
+  </si>
+  <si>
+    <t>6530-01-451-7669</t>
+  </si>
+  <si>
+    <t>U 21</t>
   </si>
 </sst>
 </file>
@@ -2719,9 +2731,13 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Items" displayName="Items" ref="A1:L215">
-  <autoFilter ref="A1:L215" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Items" displayName="Items" ref="A1:L216">
+  <autoFilter ref="A1:L216" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="category"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="shelf"/>
@@ -3025,7 +3041,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L215"/>
+  <dimension ref="A1:L216"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" style="1" customWidth="1"/>
@@ -9442,13 +9458,13 @@
         <v>782</v>
       </c>
       <c r="D195" s="3" t="s">
-        <v>783</v>
+        <v>869</v>
       </c>
       <c r="E195" s="3" t="s">
-        <v>780</v>
+        <v>870</v>
       </c>
       <c r="F195" s="3" t="s">
-        <v>784</v>
+        <v>871</v>
       </c>
       <c r="G195" s="3" t="s">
         <v>129</v>
@@ -9476,13 +9492,13 @@
         <v>785</v>
       </c>
       <c r="D196" s="3" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="E196" s="3" t="s">
-        <v>787</v>
+        <v>780</v>
       </c>
       <c r="F196" s="3" t="s">
-        <v>788</v>
+        <v>784</v>
       </c>
       <c r="G196" s="3" t="s">
         <v>129</v>
@@ -9510,29 +9526,29 @@
         <v>789</v>
       </c>
       <c r="D197" s="3" t="s">
-        <v>790</v>
+        <v>786</v>
       </c>
       <c r="E197" s="3" t="s">
-        <v>791</v>
+        <v>787</v>
       </c>
       <c r="F197" s="3" t="s">
-        <v>792</v>
+        <v>788</v>
       </c>
       <c r="G197" s="3" t="s">
-        <v>793</v>
+        <v>129</v>
       </c>
       <c r="H197" s="3" t="s">
-        <v>794</v>
+        <v>130</v>
       </c>
       <c r="I197" s="3"/>
       <c r="J197" s="3" t="s">
         <v>131</v>
       </c>
       <c r="K197" s="3" t="s">
-        <v>793</v>
+        <v>129</v>
       </c>
       <c r="L197" s="3" t="s">
-        <v>795</v>
+        <v>769</v>
       </c>
     </row>
     <row r="198" spans="1:12" x14ac:dyDescent="0.25">
@@ -9544,29 +9560,29 @@
         <v>796</v>
       </c>
       <c r="D198" s="3" t="s">
-        <v>797</v>
+        <v>790</v>
       </c>
       <c r="E198" s="3" t="s">
-        <v>798</v>
+        <v>791</v>
       </c>
       <c r="F198" s="3" t="s">
-        <v>799</v>
+        <v>792</v>
       </c>
       <c r="G198" s="3" t="s">
-        <v>264</v>
+        <v>793</v>
       </c>
       <c r="H198" s="3" t="s">
-        <v>263</v>
+        <v>794</v>
       </c>
       <c r="I198" s="3"/>
       <c r="J198" s="3" t="s">
-        <v>82</v>
+        <v>131</v>
       </c>
       <c r="K198" s="3" t="s">
-        <v>264</v>
+        <v>793</v>
       </c>
       <c r="L198" s="3" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
     </row>
     <row r="199" spans="1:12" x14ac:dyDescent="0.25">
@@ -9581,10 +9597,10 @@
         <v>797</v>
       </c>
       <c r="E199" s="3" t="s">
-        <v>587</v>
+        <v>798</v>
       </c>
       <c r="F199" s="3" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="G199" s="3" t="s">
         <v>264</v>
@@ -9612,17 +9628,19 @@
         <v>803</v>
       </c>
       <c r="D200" s="3" t="s">
-        <v>804</v>
-      </c>
-      <c r="E200" s="3"/>
+        <v>797</v>
+      </c>
+      <c r="E200" s="3" t="s">
+        <v>587</v>
+      </c>
       <c r="F200" s="3" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="G200" s="3" t="s">
         <v>264</v>
       </c>
       <c r="H200" s="3" t="s">
-        <v>446</v>
+        <v>263</v>
       </c>
       <c r="I200" s="3"/>
       <c r="J200" s="3" t="s">
@@ -9632,7 +9650,7 @@
         <v>264</v>
       </c>
       <c r="L200" s="3" t="s">
-        <v>806</v>
+        <v>800</v>
       </c>
     </row>
     <row r="201" spans="1:12" x14ac:dyDescent="0.25">
@@ -9644,29 +9662,27 @@
         <v>807</v>
       </c>
       <c r="D201" s="3" t="s">
-        <v>808</v>
-      </c>
-      <c r="E201" s="3" t="s">
-        <v>809</v>
-      </c>
+        <v>804</v>
+      </c>
+      <c r="E201" s="3"/>
       <c r="F201" s="3" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="G201" s="3" t="s">
-        <v>202</v>
+        <v>264</v>
       </c>
       <c r="H201" s="3" t="s">
-        <v>121</v>
+        <v>446</v>
       </c>
       <c r="I201" s="3"/>
       <c r="J201" s="3" t="s">
-        <v>203</v>
+        <v>82</v>
       </c>
       <c r="K201" s="3" t="s">
-        <v>202</v>
+        <v>264</v>
       </c>
       <c r="L201" s="3" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
     </row>
     <row r="202" spans="1:12" x14ac:dyDescent="0.25">
@@ -9678,29 +9694,29 @@
         <v>812</v>
       </c>
       <c r="D202" s="3" t="s">
-        <v>813</v>
+        <v>808</v>
       </c>
       <c r="E202" s="3" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
       <c r="F202" s="3" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="G202" s="3" t="s">
-        <v>816</v>
+        <v>202</v>
       </c>
       <c r="H202" s="3" t="s">
-        <v>817</v>
+        <v>121</v>
       </c>
       <c r="I202" s="3"/>
       <c r="J202" s="3" t="s">
-        <v>818</v>
+        <v>203</v>
       </c>
       <c r="K202" s="3" t="s">
-        <v>816</v>
+        <v>202</v>
       </c>
       <c r="L202" s="3" t="s">
-        <v>819</v>
+        <v>811</v>
       </c>
     </row>
     <row r="203" spans="1:12" x14ac:dyDescent="0.25">
@@ -9712,29 +9728,29 @@
         <v>820</v>
       </c>
       <c r="D203" s="3" t="s">
-        <v>821</v>
+        <v>813</v>
       </c>
       <c r="E203" s="3" t="s">
-        <v>822</v>
+        <v>814</v>
       </c>
       <c r="F203" s="3" t="s">
-        <v>823</v>
+        <v>815</v>
       </c>
       <c r="G203" s="3" t="s">
-        <v>121</v>
+        <v>816</v>
       </c>
       <c r="H203" s="3" t="s">
-        <v>121</v>
+        <v>817</v>
       </c>
       <c r="I203" s="3"/>
       <c r="J203" s="3" t="s">
-        <v>82</v>
+        <v>818</v>
       </c>
       <c r="K203" s="3" t="s">
-        <v>121</v>
+        <v>816</v>
       </c>
       <c r="L203" s="3" t="s">
-        <v>824</v>
+        <v>819</v>
       </c>
     </row>
     <row r="204" spans="1:12" x14ac:dyDescent="0.25">
@@ -9749,10 +9765,10 @@
         <v>821</v>
       </c>
       <c r="E204" s="3" t="s">
-        <v>826</v>
+        <v>822</v>
       </c>
       <c r="F204" s="3" t="s">
-        <v>827</v>
+        <v>823</v>
       </c>
       <c r="G204" s="3" t="s">
         <v>121</v>
@@ -9780,29 +9796,29 @@
         <v>828</v>
       </c>
       <c r="D205" s="3" t="s">
-        <v>829</v>
+        <v>821</v>
       </c>
       <c r="E205" s="3" t="s">
-        <v>830</v>
+        <v>826</v>
       </c>
       <c r="F205" s="3" t="s">
-        <v>831</v>
+        <v>827</v>
       </c>
       <c r="G205" s="3" t="s">
-        <v>264</v>
+        <v>121</v>
       </c>
       <c r="H205" s="3" t="s">
-        <v>446</v>
+        <v>121</v>
       </c>
       <c r="I205" s="3"/>
       <c r="J205" s="3" t="s">
         <v>82</v>
       </c>
       <c r="K205" s="3" t="s">
-        <v>264</v>
+        <v>121</v>
       </c>
       <c r="L205" s="3" t="s">
-        <v>832</v>
+        <v>824</v>
       </c>
     </row>
     <row r="206" spans="1:12" x14ac:dyDescent="0.25">
@@ -9820,7 +9836,7 @@
         <v>830</v>
       </c>
       <c r="F206" s="3" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
       <c r="G206" s="3" t="s">
         <v>264</v>
@@ -9848,29 +9864,29 @@
         <v>835</v>
       </c>
       <c r="D207" s="3" t="s">
-        <v>836</v>
+        <v>829</v>
       </c>
       <c r="E207" s="3" t="s">
-        <v>837</v>
+        <v>830</v>
       </c>
       <c r="F207" s="3" t="s">
-        <v>838</v>
+        <v>834</v>
       </c>
       <c r="G207" s="3" t="s">
-        <v>816</v>
+        <v>264</v>
       </c>
       <c r="H207" s="3" t="s">
-        <v>817</v>
+        <v>446</v>
       </c>
       <c r="I207" s="3"/>
       <c r="J207" s="3" t="s">
-        <v>818</v>
+        <v>82</v>
       </c>
       <c r="K207" s="3" t="s">
-        <v>816</v>
+        <v>264</v>
       </c>
       <c r="L207" s="3" t="s">
-        <v>819</v>
+        <v>832</v>
       </c>
     </row>
     <row r="208" spans="1:12" x14ac:dyDescent="0.25">
@@ -9882,27 +9898,29 @@
         <v>839</v>
       </c>
       <c r="D208" s="3" t="s">
-        <v>840</v>
-      </c>
-      <c r="E208" s="3"/>
+        <v>836</v>
+      </c>
+      <c r="E208" s="3" t="s">
+        <v>837</v>
+      </c>
       <c r="F208" s="3" t="s">
-        <v>841</v>
+        <v>838</v>
       </c>
       <c r="G208" s="3" t="s">
-        <v>264</v>
+        <v>816</v>
       </c>
       <c r="H208" s="3" t="s">
-        <v>263</v>
+        <v>817</v>
       </c>
       <c r="I208" s="3"/>
       <c r="J208" s="3" t="s">
-        <v>82</v>
+        <v>818</v>
       </c>
       <c r="K208" s="3" t="s">
-        <v>264</v>
+        <v>816</v>
       </c>
       <c r="L208" s="3" t="s">
-        <v>842</v>
+        <v>819</v>
       </c>
     </row>
     <row r="209" spans="1:12" x14ac:dyDescent="0.25">
@@ -9918,7 +9936,7 @@
       </c>
       <c r="E209" s="3"/>
       <c r="F209" s="3" t="s">
-        <v>844</v>
+        <v>841</v>
       </c>
       <c r="G209" s="3" t="s">
         <v>264</v>
@@ -9946,27 +9964,27 @@
         <v>845</v>
       </c>
       <c r="D210" s="3" t="s">
-        <v>846</v>
-      </c>
-      <c r="E210" s="3" t="s">
-        <v>847</v>
-      </c>
-      <c r="F210" s="3"/>
+        <v>840</v>
+      </c>
+      <c r="E210" s="3"/>
+      <c r="F210" s="3" t="s">
+        <v>844</v>
+      </c>
       <c r="G210" s="3" t="s">
-        <v>246</v>
+        <v>264</v>
       </c>
       <c r="H210" s="3" t="s">
-        <v>244</v>
+        <v>263</v>
       </c>
       <c r="I210" s="3"/>
       <c r="J210" s="3" t="s">
-        <v>245</v>
+        <v>82</v>
       </c>
       <c r="K210" s="3" t="s">
-        <v>246</v>
+        <v>264</v>
       </c>
       <c r="L210" s="3" t="s">
-        <v>848</v>
+        <v>842</v>
       </c>
     </row>
     <row r="211" spans="1:12" x14ac:dyDescent="0.25">
@@ -9975,32 +9993,30 @@
       </c>
       <c r="B211" s="3"/>
       <c r="C211" s="3" t="s">
-        <v>849</v>
+        <v>872</v>
       </c>
       <c r="D211" s="3" t="s">
-        <v>850</v>
+        <v>846</v>
       </c>
       <c r="E211" s="3" t="s">
-        <v>851</v>
-      </c>
-      <c r="F211" s="3" t="s">
-        <v>852</v>
-      </c>
+        <v>847</v>
+      </c>
+      <c r="F211" s="3"/>
       <c r="G211" s="3" t="s">
-        <v>853</v>
+        <v>246</v>
       </c>
       <c r="H211" s="3" t="s">
-        <v>817</v>
+        <v>244</v>
       </c>
       <c r="I211" s="3"/>
       <c r="J211" s="3" t="s">
-        <v>854</v>
+        <v>245</v>
       </c>
       <c r="K211" s="3" t="s">
-        <v>853</v>
+        <v>246</v>
       </c>
       <c r="L211" s="3" t="s">
-        <v>855</v>
+        <v>848</v>
       </c>
     </row>
     <row r="212" spans="1:12" x14ac:dyDescent="0.25">
@@ -10015,10 +10031,10 @@
         <v>850</v>
       </c>
       <c r="E212" s="3" t="s">
-        <v>856</v>
+        <v>851</v>
       </c>
       <c r="F212" s="3" t="s">
-        <v>857</v>
+        <v>852</v>
       </c>
       <c r="G212" s="3" t="s">
         <v>853</v>
@@ -10043,16 +10059,16 @@
       </c>
       <c r="B213" s="3"/>
       <c r="C213" s="3" t="s">
-        <v>858</v>
+        <v>849</v>
       </c>
       <c r="D213" s="3" t="s">
-        <v>859</v>
+        <v>850</v>
       </c>
       <c r="E213" s="3" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="F213" s="3" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
       <c r="G213" s="3" t="s">
         <v>853</v>
@@ -10068,7 +10084,7 @@
         <v>853</v>
       </c>
       <c r="L213" s="3" t="s">
-        <v>861</v>
+        <v>855</v>
       </c>
     </row>
     <row r="214" spans="1:12" x14ac:dyDescent="0.25">
@@ -10083,10 +10099,10 @@
         <v>859</v>
       </c>
       <c r="E214" s="3" t="s">
-        <v>856</v>
+        <v>851</v>
       </c>
       <c r="F214" s="3" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="G214" s="3" t="s">
         <v>853</v>
@@ -10111,31 +10127,65 @@
       </c>
       <c r="B215" s="3"/>
       <c r="C215" s="3" t="s">
-        <v>863</v>
+        <v>858</v>
       </c>
       <c r="D215" s="3" t="s">
-        <v>864</v>
+        <v>859</v>
       </c>
       <c r="E215" s="3" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="F215" s="3" t="s">
-        <v>865</v>
+        <v>862</v>
       </c>
       <c r="G215" s="3" t="s">
-        <v>866</v>
+        <v>853</v>
       </c>
       <c r="H215" s="3" t="s">
-        <v>866</v>
+        <v>817</v>
       </c>
       <c r="I215" s="3"/>
       <c r="J215" s="3" t="s">
+        <v>854</v>
+      </c>
+      <c r="K215" s="3" t="s">
+        <v>853</v>
+      </c>
+      <c r="L215" s="3" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="216" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A216" s="3" t="s">
+        <v>764</v>
+      </c>
+      <c r="B216" s="3"/>
+      <c r="C216" s="3" t="s">
+        <v>863</v>
+      </c>
+      <c r="D216" s="3" t="s">
+        <v>864</v>
+      </c>
+      <c r="E216" s="3" t="s">
+        <v>851</v>
+      </c>
+      <c r="F216" s="3" t="s">
+        <v>865</v>
+      </c>
+      <c r="G216" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="H216" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="I216" s="3"/>
+      <c r="J216" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="K215" s="3" t="s">
+      <c r="K216" s="3" t="s">
         <v>866</v>
       </c>
-      <c r="L215" s="3" t="s">
+      <c r="L216" s="3" t="s">
         <v>855</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Glucerna, moved male catheters
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dvagov-my.sharepoint.com/personal/bernard_chan_va_gov/Documents/Microsoft Teams Chat Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="11_87A73CECC8785890643FEBC9776139824E07390D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C7C0600-0369-45DC-AD5C-D29C9D536A08}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="11_87A73CECC8785890643FEBC9776139824E07390D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4742EE64-3A2A-4E53-BCDD-E223680C7C31}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2056" uniqueCount="873">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2066" uniqueCount="875">
   <si>
     <t>category</t>
   </si>
@@ -2655,6 +2655,12 @@
   </si>
   <si>
     <t>U 21</t>
+  </si>
+  <si>
+    <t>Glucerna Rich Chocolate</t>
+  </si>
+  <si>
+    <t>24 x 240 mL</t>
   </si>
 </sst>
 </file>
@@ -2736,8 +2742,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Items" displayName="Items" ref="A1:L216">
-  <autoFilter ref="A1:L216" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Items" displayName="Items" ref="A1:L217">
+  <autoFilter ref="A1:L217" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="category"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="shelf"/>
@@ -3041,7 +3047,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L216"/>
+  <dimension ref="A1:L217"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" style="1" customWidth="1"/>
@@ -8712,17 +8718,17 @@
         <v>690</v>
       </c>
       <c r="D173" s="3" t="s">
-        <v>698</v>
+        <v>873</v>
       </c>
       <c r="E173" s="3" t="s">
-        <v>684</v>
+        <v>874</v>
       </c>
       <c r="F173" s="3"/>
       <c r="G173" s="3" t="s">
         <v>699</v>
       </c>
       <c r="H173" s="3" t="s">
-        <v>699</v>
+        <v>685</v>
       </c>
       <c r="I173" s="3" t="s">
         <v>692</v>
@@ -8731,10 +8737,10 @@
         <v>687</v>
       </c>
       <c r="K173" s="3" t="s">
-        <v>699</v>
+        <v>685</v>
       </c>
       <c r="L173" s="3" t="s">
-        <v>700</v>
+        <v>693</v>
       </c>
     </row>
     <row r="174" spans="1:12" x14ac:dyDescent="0.25">
@@ -8746,10 +8752,10 @@
         <v>690</v>
       </c>
       <c r="D174" s="3" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="E174" s="3" t="s">
-        <v>702</v>
+        <v>684</v>
       </c>
       <c r="F174" s="3"/>
       <c r="G174" s="3" t="s">
@@ -8777,32 +8783,32 @@
       </c>
       <c r="B175" s="3"/>
       <c r="C175" s="3" t="s">
-        <v>682</v>
+        <v>690</v>
       </c>
       <c r="D175" s="3" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="E175" s="3" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="F175" s="3"/>
       <c r="G175" s="3" t="s">
-        <v>101</v>
+        <v>699</v>
       </c>
       <c r="H175" s="3" t="s">
-        <v>577</v>
+        <v>699</v>
       </c>
       <c r="I175" s="3" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
       <c r="J175" s="3" t="s">
-        <v>103</v>
+        <v>687</v>
       </c>
       <c r="K175" s="3" t="s">
-        <v>101</v>
+        <v>699</v>
       </c>
       <c r="L175" s="3" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
     </row>
     <row r="176" spans="1:12" x14ac:dyDescent="0.25">
@@ -8811,23 +8817,23 @@
       </c>
       <c r="B176" s="3"/>
       <c r="C176" s="3" t="s">
-        <v>690</v>
+        <v>682</v>
       </c>
       <c r="D176" s="3" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="E176" s="3" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="F176" s="3"/>
       <c r="G176" s="3" t="s">
         <v>101</v>
       </c>
       <c r="H176" s="3" t="s">
-        <v>102</v>
+        <v>577</v>
       </c>
       <c r="I176" s="3" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
       <c r="J176" s="3" t="s">
         <v>103</v>
@@ -8836,7 +8842,7 @@
         <v>101</v>
       </c>
       <c r="L176" s="3" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
     </row>
     <row r="177" spans="1:12" x14ac:dyDescent="0.25">
@@ -8845,23 +8851,23 @@
       </c>
       <c r="B177" s="3"/>
       <c r="C177" s="3" t="s">
-        <v>682</v>
+        <v>690</v>
       </c>
       <c r="D177" s="3" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="E177" s="3" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="F177" s="3"/>
       <c r="G177" s="3" t="s">
         <v>101</v>
       </c>
       <c r="H177" s="3" t="s">
-        <v>577</v>
+        <v>102</v>
       </c>
       <c r="I177" s="3" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
       <c r="J177" s="3" t="s">
         <v>103</v>
@@ -8870,7 +8876,7 @@
         <v>101</v>
       </c>
       <c r="L177" s="3" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
     </row>
     <row r="178" spans="1:12" x14ac:dyDescent="0.25">
@@ -8882,29 +8888,29 @@
         <v>682</v>
       </c>
       <c r="D178" s="3" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="E178" s="3" t="s">
-        <v>684</v>
+        <v>710</v>
       </c>
       <c r="F178" s="3"/>
       <c r="G178" s="3" t="s">
-        <v>685</v>
+        <v>101</v>
       </c>
       <c r="H178" s="3" t="s">
-        <v>685</v>
+        <v>577</v>
       </c>
       <c r="I178" s="3" t="s">
         <v>686</v>
       </c>
       <c r="J178" s="3" t="s">
-        <v>687</v>
+        <v>103</v>
       </c>
       <c r="K178" s="3" t="s">
-        <v>685</v>
+        <v>101</v>
       </c>
       <c r="L178" s="3" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
     </row>
     <row r="179" spans="1:12" x14ac:dyDescent="0.25">
@@ -8916,29 +8922,29 @@
         <v>682</v>
       </c>
       <c r="D179" s="3" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="E179" s="3" t="s">
-        <v>715</v>
+        <v>684</v>
       </c>
       <c r="F179" s="3"/>
       <c r="G179" s="3" t="s">
-        <v>129</v>
+        <v>685</v>
       </c>
       <c r="H179" s="3" t="s">
-        <v>716</v>
+        <v>685</v>
       </c>
       <c r="I179" s="3" t="s">
         <v>686</v>
       </c>
       <c r="J179" s="3" t="s">
-        <v>131</v>
+        <v>687</v>
       </c>
       <c r="K179" s="3" t="s">
-        <v>129</v>
+        <v>685</v>
       </c>
       <c r="L179" s="3" t="s">
-        <v>717</v>
+        <v>713</v>
       </c>
     </row>
     <row r="180" spans="1:12" x14ac:dyDescent="0.25">
@@ -8950,29 +8956,29 @@
         <v>682</v>
       </c>
       <c r="D180" s="3" t="s">
-        <v>718</v>
+        <v>714</v>
       </c>
       <c r="E180" s="3" t="s">
-        <v>719</v>
+        <v>715</v>
       </c>
       <c r="F180" s="3"/>
       <c r="G180" s="3" t="s">
-        <v>720</v>
+        <v>129</v>
       </c>
       <c r="H180" s="3" t="s">
-        <v>721</v>
+        <v>716</v>
       </c>
       <c r="I180" s="3" t="s">
         <v>686</v>
       </c>
       <c r="J180" s="3" t="s">
-        <v>722</v>
+        <v>131</v>
       </c>
       <c r="K180" s="3" t="s">
-        <v>720</v>
+        <v>129</v>
       </c>
       <c r="L180" s="3" t="s">
-        <v>723</v>
+        <v>717</v>
       </c>
     </row>
     <row r="181" spans="1:12" x14ac:dyDescent="0.25">
@@ -8984,7 +8990,7 @@
         <v>682</v>
       </c>
       <c r="D181" s="3" t="s">
-        <v>724</v>
+        <v>718</v>
       </c>
       <c r="E181" s="3" t="s">
         <v>719</v>
@@ -9018,29 +9024,29 @@
         <v>682</v>
       </c>
       <c r="D182" s="3" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E182" s="3" t="s">
-        <v>684</v>
+        <v>719</v>
       </c>
       <c r="F182" s="3"/>
       <c r="G182" s="3" t="s">
-        <v>685</v>
+        <v>720</v>
       </c>
       <c r="H182" s="3" t="s">
-        <v>685</v>
+        <v>721</v>
       </c>
       <c r="I182" s="3" t="s">
         <v>686</v>
       </c>
       <c r="J182" s="3" t="s">
-        <v>687</v>
+        <v>722</v>
       </c>
       <c r="K182" s="3" t="s">
-        <v>685</v>
+        <v>720</v>
       </c>
       <c r="L182" s="3" t="s">
-        <v>713</v>
+        <v>723</v>
       </c>
     </row>
     <row r="183" spans="1:12" x14ac:dyDescent="0.25">
@@ -9052,63 +9058,63 @@
         <v>682</v>
       </c>
       <c r="D183" s="3" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E183" s="3" t="s">
-        <v>727</v>
+        <v>684</v>
       </c>
       <c r="F183" s="3"/>
       <c r="G183" s="3" t="s">
-        <v>728</v>
+        <v>685</v>
       </c>
       <c r="H183" s="3" t="s">
-        <v>729</v>
+        <v>685</v>
       </c>
       <c r="I183" s="3" t="s">
         <v>686</v>
       </c>
       <c r="J183" s="3" t="s">
-        <v>730</v>
+        <v>687</v>
       </c>
       <c r="K183" s="3" t="s">
-        <v>728</v>
+        <v>685</v>
       </c>
       <c r="L183" s="3" t="s">
-        <v>731</v>
+        <v>713</v>
       </c>
     </row>
     <row r="184" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A184" s="3" t="s">
-        <v>732</v>
+        <v>681</v>
       </c>
       <c r="B184" s="3"/>
       <c r="C184" s="3" t="s">
-        <v>733</v>
+        <v>682</v>
       </c>
       <c r="D184" s="3" t="s">
-        <v>734</v>
+        <v>726</v>
       </c>
       <c r="E184" s="3" t="s">
-        <v>735</v>
-      </c>
-      <c r="F184" s="3" t="s">
-        <v>736</v>
-      </c>
+        <v>727</v>
+      </c>
+      <c r="F184" s="3"/>
       <c r="G184" s="3" t="s">
-        <v>737</v>
+        <v>728</v>
       </c>
       <c r="H184" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="I184" s="3"/>
+        <v>729</v>
+      </c>
+      <c r="I184" s="3" t="s">
+        <v>686</v>
+      </c>
       <c r="J184" s="3" t="s">
-        <v>738</v>
+        <v>730</v>
       </c>
       <c r="K184" s="3" t="s">
-        <v>737</v>
+        <v>728</v>
       </c>
       <c r="L184" s="3" t="s">
-        <v>739</v>
+        <v>731</v>
       </c>
     </row>
     <row r="185" spans="1:12" x14ac:dyDescent="0.25">
@@ -9117,32 +9123,32 @@
       </c>
       <c r="B185" s="3"/>
       <c r="C185" s="3" t="s">
-        <v>740</v>
+        <v>733</v>
       </c>
       <c r="D185" s="3" t="s">
-        <v>741</v>
+        <v>734</v>
       </c>
       <c r="E185" s="3" t="s">
-        <v>742</v>
+        <v>735</v>
       </c>
       <c r="F185" s="3" t="s">
-        <v>743</v>
+        <v>736</v>
       </c>
       <c r="G185" s="3" t="s">
-        <v>121</v>
+        <v>737</v>
       </c>
       <c r="H185" s="3" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I185" s="3"/>
       <c r="J185" s="3" t="s">
-        <v>82</v>
+        <v>738</v>
       </c>
       <c r="K185" s="3" t="s">
-        <v>121</v>
+        <v>737</v>
       </c>
       <c r="L185" s="3" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
     </row>
     <row r="186" spans="1:12" x14ac:dyDescent="0.25">
@@ -9151,32 +9157,32 @@
       </c>
       <c r="B186" s="3"/>
       <c r="C186" s="3" t="s">
-        <v>745</v>
+        <v>740</v>
       </c>
       <c r="D186" s="3" t="s">
-        <v>746</v>
+        <v>741</v>
       </c>
       <c r="E186" s="3" t="s">
-        <v>319</v>
+        <v>742</v>
       </c>
       <c r="F186" s="3" t="s">
-        <v>747</v>
+        <v>743</v>
       </c>
       <c r="G186" s="3" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="H186" s="3" t="s">
-        <v>716</v>
+        <v>121</v>
       </c>
       <c r="I186" s="3"/>
       <c r="J186" s="3" t="s">
-        <v>131</v>
+        <v>82</v>
       </c>
       <c r="K186" s="3" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="L186" s="3" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
     </row>
     <row r="187" spans="1:12" x14ac:dyDescent="0.25">
@@ -9185,32 +9191,32 @@
       </c>
       <c r="B187" s="3"/>
       <c r="C187" s="3" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="D187" s="3" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
       <c r="E187" s="3" t="s">
-        <v>751</v>
+        <v>319</v>
       </c>
       <c r="F187" s="3" t="s">
-        <v>752</v>
+        <v>747</v>
       </c>
       <c r="G187" s="3" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="H187" s="3" t="s">
-        <v>135</v>
+        <v>716</v>
       </c>
       <c r="I187" s="3"/>
       <c r="J187" s="3" t="s">
-        <v>82</v>
+        <v>131</v>
       </c>
       <c r="K187" s="3" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="L187" s="3" t="s">
-        <v>753</v>
+        <v>748</v>
       </c>
     </row>
     <row r="188" spans="1:12" x14ac:dyDescent="0.25">
@@ -9219,16 +9225,16 @@
       </c>
       <c r="B188" s="3"/>
       <c r="C188" s="3" t="s">
-        <v>754</v>
+        <v>749</v>
       </c>
       <c r="D188" s="3" t="s">
-        <v>755</v>
+        <v>750</v>
       </c>
       <c r="E188" s="3" t="s">
-        <v>756</v>
+        <v>751</v>
       </c>
       <c r="F188" s="3" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="G188" s="3" t="s">
         <v>135</v>
@@ -9244,7 +9250,7 @@
         <v>135</v>
       </c>
       <c r="L188" s="3" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
     </row>
     <row r="189" spans="1:12" x14ac:dyDescent="0.25">
@@ -9253,16 +9259,16 @@
       </c>
       <c r="B189" s="3"/>
       <c r="C189" s="3" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="D189" s="3" t="s">
         <v>755</v>
       </c>
       <c r="E189" s="3" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="F189" s="3" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="G189" s="3" t="s">
         <v>135</v>
@@ -9287,64 +9293,64 @@
       </c>
       <c r="B190" s="3"/>
       <c r="C190" s="3" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="D190" s="3" t="s">
-        <v>761</v>
-      </c>
-      <c r="E190" s="3"/>
+        <v>755</v>
+      </c>
+      <c r="E190" s="3" t="s">
+        <v>759</v>
+      </c>
       <c r="F190" s="3" t="s">
-        <v>762</v>
+        <v>759</v>
       </c>
       <c r="G190" s="3" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="H190" s="3" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="I190" s="3"/>
       <c r="J190" s="3" t="s">
         <v>82</v>
       </c>
       <c r="K190" s="3" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="L190" s="3" t="s">
-        <v>763</v>
+        <v>757</v>
       </c>
     </row>
     <row r="191" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A191" s="3" t="s">
-        <v>764</v>
+        <v>732</v>
       </c>
       <c r="B191" s="3"/>
       <c r="C191" s="3" t="s">
-        <v>765</v>
+        <v>760</v>
       </c>
       <c r="D191" s="3" t="s">
-        <v>766</v>
-      </c>
-      <c r="E191" s="3" t="s">
-        <v>767</v>
-      </c>
+        <v>761</v>
+      </c>
+      <c r="E191" s="3"/>
       <c r="F191" s="3" t="s">
-        <v>768</v>
+        <v>762</v>
       </c>
       <c r="G191" s="3" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="H191" s="3" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="I191" s="3"/>
       <c r="J191" s="3" t="s">
-        <v>131</v>
+        <v>82</v>
       </c>
       <c r="K191" s="3" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="L191" s="3" t="s">
-        <v>769</v>
+        <v>763</v>
       </c>
     </row>
     <row r="192" spans="1:12" x14ac:dyDescent="0.25">
@@ -9353,29 +9359,29 @@
       </c>
       <c r="B192" s="3"/>
       <c r="C192" s="3" t="s">
-        <v>770</v>
+        <v>765</v>
       </c>
       <c r="D192" s="3" t="s">
-        <v>771</v>
+        <v>766</v>
       </c>
       <c r="E192" s="3" t="s">
-        <v>772</v>
+        <v>767</v>
       </c>
       <c r="F192" s="3" t="s">
-        <v>773</v>
+        <v>768</v>
       </c>
       <c r="G192" s="3" t="s">
-        <v>17</v>
+        <v>129</v>
       </c>
       <c r="H192" s="3" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="I192" s="3"/>
       <c r="J192" s="3" t="s">
-        <v>18</v>
+        <v>131</v>
       </c>
       <c r="K192" s="3" t="s">
-        <v>17</v>
+        <v>129</v>
       </c>
       <c r="L192" s="3" t="s">
         <v>769</v>
@@ -9387,16 +9393,16 @@
       </c>
       <c r="B193" s="3"/>
       <c r="C193" s="3" t="s">
-        <v>774</v>
+        <v>770</v>
       </c>
       <c r="D193" s="3" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
       <c r="E193" s="3" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="F193" s="3" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="G193" s="3" t="s">
         <v>17</v>
@@ -9421,29 +9427,29 @@
       </c>
       <c r="B194" s="3"/>
       <c r="C194" s="3" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="D194" s="3" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="E194" s="3" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="F194" s="3" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="G194" s="3" t="s">
-        <v>129</v>
+        <v>17</v>
       </c>
       <c r="H194" s="3" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="I194" s="3"/>
       <c r="J194" s="3" t="s">
-        <v>131</v>
+        <v>18</v>
       </c>
       <c r="K194" s="3" t="s">
-        <v>129</v>
+        <v>17</v>
       </c>
       <c r="L194" s="3" t="s">
         <v>769</v>
@@ -9455,16 +9461,16 @@
       </c>
       <c r="B195" s="3"/>
       <c r="C195" s="3" t="s">
-        <v>782</v>
+        <v>778</v>
       </c>
       <c r="D195" s="3" t="s">
-        <v>783</v>
+        <v>869</v>
       </c>
       <c r="E195" s="3" t="s">
-        <v>780</v>
+        <v>870</v>
       </c>
       <c r="F195" s="3" t="s">
-        <v>784</v>
+        <v>871</v>
       </c>
       <c r="G195" s="3" t="s">
         <v>129</v>
@@ -9489,16 +9495,16 @@
       </c>
       <c r="B196" s="3"/>
       <c r="C196" s="3" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="D196" s="3" t="s">
-        <v>869</v>
+        <v>779</v>
       </c>
       <c r="E196" s="3" t="s">
-        <v>870</v>
+        <v>780</v>
       </c>
       <c r="F196" s="3" t="s">
-        <v>871</v>
+        <v>781</v>
       </c>
       <c r="G196" s="3" t="s">
         <v>129</v>
@@ -9523,16 +9529,16 @@
       </c>
       <c r="B197" s="3"/>
       <c r="C197" s="3" t="s">
-        <v>789</v>
+        <v>785</v>
       </c>
       <c r="D197" s="3" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="E197" s="3" t="s">
-        <v>787</v>
+        <v>780</v>
       </c>
       <c r="F197" s="3" t="s">
-        <v>788</v>
+        <v>784</v>
       </c>
       <c r="G197" s="3" t="s">
         <v>129</v>
@@ -9557,32 +9563,32 @@
       </c>
       <c r="B198" s="3"/>
       <c r="C198" s="3" t="s">
-        <v>796</v>
+        <v>789</v>
       </c>
       <c r="D198" s="3" t="s">
-        <v>790</v>
+        <v>786</v>
       </c>
       <c r="E198" s="3" t="s">
-        <v>791</v>
+        <v>787</v>
       </c>
       <c r="F198" s="3" t="s">
-        <v>792</v>
+        <v>788</v>
       </c>
       <c r="G198" s="3" t="s">
-        <v>793</v>
+        <v>129</v>
       </c>
       <c r="H198" s="3" t="s">
-        <v>794</v>
+        <v>130</v>
       </c>
       <c r="I198" s="3"/>
       <c r="J198" s="3" t="s">
         <v>131</v>
       </c>
       <c r="K198" s="3" t="s">
-        <v>793</v>
+        <v>129</v>
       </c>
       <c r="L198" s="3" t="s">
-        <v>795</v>
+        <v>769</v>
       </c>
     </row>
     <row r="199" spans="1:12" x14ac:dyDescent="0.25">
@@ -9591,32 +9597,32 @@
       </c>
       <c r="B199" s="3"/>
       <c r="C199" s="3" t="s">
-        <v>801</v>
+        <v>796</v>
       </c>
       <c r="D199" s="3" t="s">
-        <v>797</v>
+        <v>790</v>
       </c>
       <c r="E199" s="3" t="s">
-        <v>798</v>
+        <v>791</v>
       </c>
       <c r="F199" s="3" t="s">
-        <v>799</v>
+        <v>792</v>
       </c>
       <c r="G199" s="3" t="s">
-        <v>264</v>
+        <v>793</v>
       </c>
       <c r="H199" s="3" t="s">
-        <v>263</v>
+        <v>794</v>
       </c>
       <c r="I199" s="3"/>
       <c r="J199" s="3" t="s">
-        <v>82</v>
+        <v>131</v>
       </c>
       <c r="K199" s="3" t="s">
-        <v>264</v>
+        <v>793</v>
       </c>
       <c r="L199" s="3" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
     </row>
     <row r="200" spans="1:12" x14ac:dyDescent="0.25">
@@ -9625,16 +9631,16 @@
       </c>
       <c r="B200" s="3"/>
       <c r="C200" s="3" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="D200" s="3" t="s">
         <v>797</v>
       </c>
       <c r="E200" s="3" t="s">
-        <v>587</v>
+        <v>798</v>
       </c>
       <c r="F200" s="3" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="G200" s="3" t="s">
         <v>264</v>
@@ -9659,20 +9665,22 @@
       </c>
       <c r="B201" s="3"/>
       <c r="C201" s="3" t="s">
-        <v>807</v>
+        <v>803</v>
       </c>
       <c r="D201" s="3" t="s">
-        <v>804</v>
-      </c>
-      <c r="E201" s="3"/>
+        <v>797</v>
+      </c>
+      <c r="E201" s="3" t="s">
+        <v>587</v>
+      </c>
       <c r="F201" s="3" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="G201" s="3" t="s">
         <v>264</v>
       </c>
       <c r="H201" s="3" t="s">
-        <v>446</v>
+        <v>263</v>
       </c>
       <c r="I201" s="3"/>
       <c r="J201" s="3" t="s">
@@ -9682,7 +9690,7 @@
         <v>264</v>
       </c>
       <c r="L201" s="3" t="s">
-        <v>806</v>
+        <v>800</v>
       </c>
     </row>
     <row r="202" spans="1:12" x14ac:dyDescent="0.25">
@@ -9691,32 +9699,30 @@
       </c>
       <c r="B202" s="3"/>
       <c r="C202" s="3" t="s">
-        <v>812</v>
+        <v>807</v>
       </c>
       <c r="D202" s="3" t="s">
-        <v>808</v>
-      </c>
-      <c r="E202" s="3" t="s">
-        <v>809</v>
-      </c>
+        <v>804</v>
+      </c>
+      <c r="E202" s="3"/>
       <c r="F202" s="3" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="G202" s="3" t="s">
-        <v>202</v>
+        <v>264</v>
       </c>
       <c r="H202" s="3" t="s">
-        <v>121</v>
+        <v>446</v>
       </c>
       <c r="I202" s="3"/>
       <c r="J202" s="3" t="s">
-        <v>203</v>
+        <v>82</v>
       </c>
       <c r="K202" s="3" t="s">
-        <v>202</v>
+        <v>264</v>
       </c>
       <c r="L202" s="3" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
     </row>
     <row r="203" spans="1:12" x14ac:dyDescent="0.25">
@@ -9725,32 +9731,32 @@
       </c>
       <c r="B203" s="3"/>
       <c r="C203" s="3" t="s">
-        <v>820</v>
+        <v>812</v>
       </c>
       <c r="D203" s="3" t="s">
-        <v>813</v>
+        <v>808</v>
       </c>
       <c r="E203" s="3" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
       <c r="F203" s="3" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="G203" s="3" t="s">
-        <v>816</v>
+        <v>202</v>
       </c>
       <c r="H203" s="3" t="s">
-        <v>817</v>
+        <v>121</v>
       </c>
       <c r="I203" s="3"/>
       <c r="J203" s="3" t="s">
-        <v>818</v>
+        <v>203</v>
       </c>
       <c r="K203" s="3" t="s">
-        <v>816</v>
+        <v>202</v>
       </c>
       <c r="L203" s="3" t="s">
-        <v>819</v>
+        <v>811</v>
       </c>
     </row>
     <row r="204" spans="1:12" x14ac:dyDescent="0.25">
@@ -9759,32 +9765,32 @@
       </c>
       <c r="B204" s="3"/>
       <c r="C204" s="3" t="s">
-        <v>825</v>
+        <v>820</v>
       </c>
       <c r="D204" s="3" t="s">
-        <v>821</v>
+        <v>813</v>
       </c>
       <c r="E204" s="3" t="s">
-        <v>822</v>
+        <v>814</v>
       </c>
       <c r="F204" s="3" t="s">
-        <v>823</v>
+        <v>815</v>
       </c>
       <c r="G204" s="3" t="s">
-        <v>121</v>
+        <v>816</v>
       </c>
       <c r="H204" s="3" t="s">
-        <v>121</v>
+        <v>817</v>
       </c>
       <c r="I204" s="3"/>
       <c r="J204" s="3" t="s">
-        <v>82</v>
+        <v>818</v>
       </c>
       <c r="K204" s="3" t="s">
-        <v>121</v>
+        <v>816</v>
       </c>
       <c r="L204" s="3" t="s">
-        <v>824</v>
+        <v>819</v>
       </c>
     </row>
     <row r="205" spans="1:12" x14ac:dyDescent="0.25">
@@ -9793,16 +9799,16 @@
       </c>
       <c r="B205" s="3"/>
       <c r="C205" s="3" t="s">
-        <v>828</v>
+        <v>825</v>
       </c>
       <c r="D205" s="3" t="s">
         <v>821</v>
       </c>
       <c r="E205" s="3" t="s">
-        <v>826</v>
+        <v>822</v>
       </c>
       <c r="F205" s="3" t="s">
-        <v>827</v>
+        <v>823</v>
       </c>
       <c r="G205" s="3" t="s">
         <v>121</v>
@@ -9827,32 +9833,32 @@
       </c>
       <c r="B206" s="3"/>
       <c r="C206" s="3" t="s">
-        <v>833</v>
+        <v>828</v>
       </c>
       <c r="D206" s="3" t="s">
-        <v>829</v>
+        <v>821</v>
       </c>
       <c r="E206" s="3" t="s">
-        <v>830</v>
+        <v>826</v>
       </c>
       <c r="F206" s="3" t="s">
-        <v>831</v>
+        <v>827</v>
       </c>
       <c r="G206" s="3" t="s">
-        <v>264</v>
+        <v>121</v>
       </c>
       <c r="H206" s="3" t="s">
-        <v>446</v>
+        <v>121</v>
       </c>
       <c r="I206" s="3"/>
       <c r="J206" s="3" t="s">
         <v>82</v>
       </c>
       <c r="K206" s="3" t="s">
-        <v>264</v>
+        <v>121</v>
       </c>
       <c r="L206" s="3" t="s">
-        <v>832</v>
+        <v>824</v>
       </c>
     </row>
     <row r="207" spans="1:12" x14ac:dyDescent="0.25">
@@ -9861,7 +9867,7 @@
       </c>
       <c r="B207" s="3"/>
       <c r="C207" s="3" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="D207" s="3" t="s">
         <v>829</v>
@@ -9870,7 +9876,7 @@
         <v>830</v>
       </c>
       <c r="F207" s="3" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
       <c r="G207" s="3" t="s">
         <v>264</v>
@@ -9895,32 +9901,32 @@
       </c>
       <c r="B208" s="3"/>
       <c r="C208" s="3" t="s">
-        <v>839</v>
+        <v>835</v>
       </c>
       <c r="D208" s="3" t="s">
-        <v>836</v>
+        <v>829</v>
       </c>
       <c r="E208" s="3" t="s">
-        <v>837</v>
+        <v>830</v>
       </c>
       <c r="F208" s="3" t="s">
-        <v>838</v>
+        <v>834</v>
       </c>
       <c r="G208" s="3" t="s">
-        <v>816</v>
+        <v>264</v>
       </c>
       <c r="H208" s="3" t="s">
-        <v>817</v>
+        <v>446</v>
       </c>
       <c r="I208" s="3"/>
       <c r="J208" s="3" t="s">
-        <v>818</v>
+        <v>82</v>
       </c>
       <c r="K208" s="3" t="s">
-        <v>816</v>
+        <v>264</v>
       </c>
       <c r="L208" s="3" t="s">
-        <v>819</v>
+        <v>832</v>
       </c>
     </row>
     <row r="209" spans="1:12" x14ac:dyDescent="0.25">
@@ -9929,30 +9935,32 @@
       </c>
       <c r="B209" s="3"/>
       <c r="C209" s="3" t="s">
-        <v>843</v>
+        <v>839</v>
       </c>
       <c r="D209" s="3" t="s">
-        <v>840</v>
-      </c>
-      <c r="E209" s="3"/>
+        <v>836</v>
+      </c>
+      <c r="E209" s="3" t="s">
+        <v>837</v>
+      </c>
       <c r="F209" s="3" t="s">
-        <v>841</v>
+        <v>838</v>
       </c>
       <c r="G209" s="3" t="s">
-        <v>264</v>
+        <v>816</v>
       </c>
       <c r="H209" s="3" t="s">
-        <v>263</v>
+        <v>817</v>
       </c>
       <c r="I209" s="3"/>
       <c r="J209" s="3" t="s">
-        <v>82</v>
+        <v>818</v>
       </c>
       <c r="K209" s="3" t="s">
-        <v>264</v>
+        <v>816</v>
       </c>
       <c r="L209" s="3" t="s">
-        <v>842</v>
+        <v>819</v>
       </c>
     </row>
     <row r="210" spans="1:12" x14ac:dyDescent="0.25">
@@ -9961,14 +9969,14 @@
       </c>
       <c r="B210" s="3"/>
       <c r="C210" s="3" t="s">
-        <v>845</v>
+        <v>843</v>
       </c>
       <c r="D210" s="3" t="s">
         <v>840</v>
       </c>
       <c r="E210" s="3"/>
       <c r="F210" s="3" t="s">
-        <v>844</v>
+        <v>841</v>
       </c>
       <c r="G210" s="3" t="s">
         <v>264</v>
@@ -9993,30 +10001,30 @@
       </c>
       <c r="B211" s="3"/>
       <c r="C211" s="3" t="s">
-        <v>872</v>
+        <v>845</v>
       </c>
       <c r="D211" s="3" t="s">
-        <v>846</v>
-      </c>
-      <c r="E211" s="3" t="s">
-        <v>847</v>
-      </c>
-      <c r="F211" s="3"/>
+        <v>840</v>
+      </c>
+      <c r="E211" s="3"/>
+      <c r="F211" s="3" t="s">
+        <v>844</v>
+      </c>
       <c r="G211" s="3" t="s">
-        <v>246</v>
+        <v>264</v>
       </c>
       <c r="H211" s="3" t="s">
-        <v>244</v>
+        <v>263</v>
       </c>
       <c r="I211" s="3"/>
       <c r="J211" s="3" t="s">
-        <v>245</v>
+        <v>82</v>
       </c>
       <c r="K211" s="3" t="s">
-        <v>246</v>
+        <v>264</v>
       </c>
       <c r="L211" s="3" t="s">
-        <v>848</v>
+        <v>842</v>
       </c>
     </row>
     <row r="212" spans="1:12" x14ac:dyDescent="0.25">
@@ -10025,32 +10033,30 @@
       </c>
       <c r="B212" s="3"/>
       <c r="C212" s="3" t="s">
-        <v>849</v>
+        <v>872</v>
       </c>
       <c r="D212" s="3" t="s">
-        <v>850</v>
+        <v>846</v>
       </c>
       <c r="E212" s="3" t="s">
-        <v>851</v>
-      </c>
-      <c r="F212" s="3" t="s">
-        <v>852</v>
-      </c>
+        <v>847</v>
+      </c>
+      <c r="F212" s="3"/>
       <c r="G212" s="3" t="s">
-        <v>853</v>
+        <v>246</v>
       </c>
       <c r="H212" s="3" t="s">
-        <v>817</v>
+        <v>244</v>
       </c>
       <c r="I212" s="3"/>
       <c r="J212" s="3" t="s">
-        <v>854</v>
+        <v>245</v>
       </c>
       <c r="K212" s="3" t="s">
-        <v>853</v>
+        <v>246</v>
       </c>
       <c r="L212" s="3" t="s">
-        <v>855</v>
+        <v>848</v>
       </c>
     </row>
     <row r="213" spans="1:12" x14ac:dyDescent="0.25">
@@ -10065,10 +10071,10 @@
         <v>850</v>
       </c>
       <c r="E213" s="3" t="s">
-        <v>856</v>
+        <v>851</v>
       </c>
       <c r="F213" s="3" t="s">
-        <v>857</v>
+        <v>852</v>
       </c>
       <c r="G213" s="3" t="s">
         <v>853</v>
@@ -10093,16 +10099,16 @@
       </c>
       <c r="B214" s="3"/>
       <c r="C214" s="3" t="s">
-        <v>858</v>
+        <v>849</v>
       </c>
       <c r="D214" s="3" t="s">
-        <v>859</v>
+        <v>850</v>
       </c>
       <c r="E214" s="3" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="F214" s="3" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
       <c r="G214" s="3" t="s">
         <v>853</v>
@@ -10118,7 +10124,7 @@
         <v>853</v>
       </c>
       <c r="L214" s="3" t="s">
-        <v>861</v>
+        <v>855</v>
       </c>
     </row>
     <row r="215" spans="1:12" x14ac:dyDescent="0.25">
@@ -10133,10 +10139,10 @@
         <v>859</v>
       </c>
       <c r="E215" s="3" t="s">
-        <v>856</v>
+        <v>851</v>
       </c>
       <c r="F215" s="3" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="G215" s="3" t="s">
         <v>853</v>
@@ -10161,31 +10167,65 @@
       </c>
       <c r="B216" s="3"/>
       <c r="C216" s="3" t="s">
-        <v>863</v>
+        <v>858</v>
       </c>
       <c r="D216" s="3" t="s">
-        <v>864</v>
+        <v>859</v>
       </c>
       <c r="E216" s="3" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="F216" s="3" t="s">
-        <v>865</v>
+        <v>862</v>
       </c>
       <c r="G216" s="3" t="s">
-        <v>866</v>
+        <v>853</v>
       </c>
       <c r="H216" s="3" t="s">
-        <v>866</v>
+        <v>817</v>
       </c>
       <c r="I216" s="3"/>
       <c r="J216" s="3" t="s">
+        <v>854</v>
+      </c>
+      <c r="K216" s="3" t="s">
+        <v>853</v>
+      </c>
+      <c r="L216" s="3" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="217" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A217" s="3" t="s">
+        <v>764</v>
+      </c>
+      <c r="B217" s="3"/>
+      <c r="C217" s="3" t="s">
+        <v>863</v>
+      </c>
+      <c r="D217" s="3" t="s">
+        <v>864</v>
+      </c>
+      <c r="E217" s="3" t="s">
+        <v>851</v>
+      </c>
+      <c r="F217" s="3" t="s">
+        <v>865</v>
+      </c>
+      <c r="G217" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="H217" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="I217" s="3"/>
+      <c r="J217" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="K216" s="3" t="s">
+      <c r="K217" s="3" t="s">
         <v>866</v>
       </c>
-      <c r="L216" s="3" t="s">
+      <c r="L217" s="3" t="s">
         <v>855</v>
       </c>
     </row>

</xml_diff>